<commit_message>
i forgot what i changed
</commit_message>
<xml_diff>
--- a/PCB/materials.xlsx
+++ b/PCB/materials.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joshf\Documents\Code\USB_IR_Blaster\PCB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A4E20FE-3077-48BE-94DA-8CE92E0E62BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9814267-C47A-47AD-83EE-FF15C4386B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{FC31D8FB-3664-43EE-8E32-81502E5E38D7}"/>
   </bookViews>
@@ -242,13 +242,13 @@
     <t>Button_Switch_SMD:SW_Push_6x3.5mm</t>
   </si>
   <si>
-    <t>STDCRG1-12M</t>
-  </si>
-  <si>
     <t>https://www.mouser.com/ProductDetail/ABRACON/ABM8-272-T3?qs=QpmGXVUTftEj6miOiJBMxQ%3D%3D&amp;srsltid=AfmBOoreONVOH-K9twHGfSJF-Jpo5aXiXpnElmP-T8XmVjeTsv9DHJFU</t>
   </si>
   <si>
     <t>Crystals Ultra Miniature Ceramic SMD Crystal</t>
+  </si>
+  <si>
+    <t>ABM8-272-T3</t>
   </si>
 </sst>
 </file>
@@ -916,13 +916,13 @@
     </row>
     <row r="14" spans="1:8" ht="213.75" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" t="s">
         <v>69</v>
       </c>
-      <c r="C14" t="s">
+      <c r="E14" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>